<commit_message>
feat(umsetzung): Schema-Attribute auslesen statt Attributnamen raten
Für die 14a-Strecke fehlt der Mapping-Vorschlag - Billing hat nur
Einspeiser zugeordnet. Statt Attributnamen zu erfinden, liest das neue
Werkzeug sie aus dem konfigurierten Schema.

tools/schema_attribute.py:
- listet alle Attribute eines Schemas (Name, Label, Typ, Pflicht, Gruppe,
  Auswahloptionen) über GET /v1/entity/schemas/{slug}
- ordnet optional eine Spaltenliste nach Namensähnlichkeit zu und gibt bis
  zu drei Vorschläge je Spalte mit Gütewert aus
- löst dabei die Abkürzungen der Exportspalten auf (WP, SP, ZN, ZS, IBN,
  AB, AO), sonst greift kein Vergleich

Die Vorschläge sind ausdrücklich ungeprüft und ein Startpunkt für die
Runde, keine Entscheidung. In der Arbeitsmappe ist vermerkt, dass die
Spalte "Quelle in epilot" bewusst leer ist und wie sie zu füllen ist.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZbuP36KCGaT5y7SLsajDV
</commit_message>
<xml_diff>
--- a/besprechung/Mapping-Sitzung_14a.xlsx
+++ b/besprechung/Mapping-Sitzung_14a.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,6 +121,12 @@
       <color rgb="004A5A63"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005A6A73"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -186,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -251,6 +257,7 @@
     <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -853,7 +860,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Gelb ausfüllen. „Anzeige?“ = vermutlich reiner Formulartext — erst Entscheidung 1 klären.</t>
+          <t>Die Spalte "Quelle in epilot" ist bewusst leer: Für § 14a liegt noch kein Mapping-Vorschlag vor (Billing hat nur die Einspeiser-Strecke zugeordnet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Vorschläge erzeugen statt raten: umsetzung/tools/schema_attribute.py liest die Attribute des epilot-Schemas aus und ordnet sie den Spalten nach Namensähnlichkeit zu.</t>
         </is>
       </c>
     </row>

</xml_diff>